<commit_message>
feat(itrust-study): publish specification and test suite v3.0
</commit_message>
<xml_diff>
--- a/output/xlsx/UC1UserFunctionality--GT-.xlsx
+++ b/output/xlsx/UC1UserFunctionality--GT-.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Version: </t>
   </si>
   <si>
-    <t>2.0</t>
+    <t>3.0</t>
   </si>
   <si>
     <t>Suite Type:</t>
@@ -92,7 +92,7 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>admin: An Admin enters a user name, a password, confirm password, the role, and if the user is enabled (or active) in the system. The Admin presses the button to add the user . The user name serves as the User's Medical ID (MID). The possible roles are: Patient Health Care Provider (HCP) Admin</t>
+    <t>admin: An Admin enters a user name, a password, confirm password, the role, and if the user is enabled (or active) in the system. The Admin presses the button to add the user . The user name serves as the User's Medical ID (MID). The possible roles are: Patient Health Care Provider (HCP) Admin Emergency Responder (ER) Lab Tech</t>
   </si>
   <si>
     <t/>
@@ -230,7 +230,7 @@
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="17.578125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="238.1875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="255.0" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="21.8984375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="124.33984375" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="30.5234375" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
feat(itrust-study): publish specification and test suite v4.0
</commit_message>
<xml_diff>
--- a/output/xlsx/UC1UserFunctionality--GT-.xlsx
+++ b/output/xlsx/UC1UserFunctionality--GT-.xlsx
@@ -29,7 +29,7 @@
     <t xml:space="preserve">Version: </t>
   </si>
   <si>
-    <t>3.0</t>
+    <t>4.0</t>
   </si>
   <si>
     <t>Suite Type:</t>
@@ -92,7 +92,7 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>admin: An Admin enters a user name, a password, confirm password, the role, and if the user is enabled (or active) in the system. The Admin presses the button to add the user . The user name serves as the User's Medical ID (MID). The possible roles are: Patient Health Care Provider (HCP) Admin Emergency Responder (ER) Lab Tech</t>
+    <t>admin: An Admin enters a user name, a password, confirm password, the role, and if the user is enabled (or active) in the system. The Admin presses the button to add the user . The user name serves as the User's Medical ID (MID). The possible roles are: Patient Health Care Provider (HCP) Optometrist HCP Ophthalmologist HCP Admin Emergency Responder (ER) Lab Tech</t>
   </si>
   <si>
     <t/>

</xml_diff>